<commit_message>
Added descriptions and added sorting method.
</commit_message>
<xml_diff>
--- a/public/Art_Courses.xlsx
+++ b/public/Art_Courses.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CJ\Documents\My Projects\Spectrum Works Projects\photoshop-courses\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CJ\Documents\My Projects\Spectrum Works Projects\art-courses\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EF152F2-9F66-4BAD-912E-F41CBA05BEB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68889C94-2002-4FCC-B869-D2B9B222FD81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Photoshop" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="176">
   <si>
     <t>ID</t>
   </si>
@@ -499,16 +499,10 @@
     <t>Basics of Animation</t>
   </si>
   <si>
-    <t>https://www.udemy.com/course/begin-animation/?utm_campaign=Search_DSA_Beta_Prof_la.EN_cc.US&amp;utm_source=google&amp;utm_medium=paid-search&amp;portfolio=USA&amp;utm_audience=mx&amp;utm_tactic=nb&amp;utm_term=_._ag_162107351473_._ad_696074114859_._kw_&amp;utm_content=g&amp;funnel=&amp;test=&amp;campaignid=21164973268&amp;adgroupid=162107351473&amp;device=c&amp;keyword=&amp;matchtype=&amp;network=g&amp;devicemodel=&amp;creativeid=696074114859&amp;assetgroupid=&amp;targetid=aud-1748515510702%3Adsa-2435203043973&amp;extensionid=&amp;placement=&amp;gad_source=1&amp;gad_campaignid=21164973268&amp;gbraid=0AAAAADROdO3vV3srGaLnx8wKT1ORyb2GY&amp;gclid=Cj0KCQjwnbrUBhDOARIsAKKhPpdRt5LScRL_ACtHKBxygXyQvQ412VeQAYV3I2zhz1xdaxIBluI9rSgaAst-EALw_wcB&amp;couponCode=CP260817G1</t>
-  </si>
-  <si>
     <t>This course is perfect if you want to pursue a career in animation and you have never animated before.</t>
   </si>
   <si>
     <t>$13/month</t>
-  </si>
-  <si>
-    <t>https://www.udemy.com/course/learn-animation/?couponCode=CP260817G1</t>
   </si>
   <si>
     <t>Learn How to Animate: 2D Animation for Beginners</t>
@@ -621,6 +615,77 @@
   </si>
   <si>
     <t>https://www.nobledesktop.com/seminars/intro-after-effects</t>
+  </si>
+  <si>
+    <t>https://www.udemy.com/course/begin-animation</t>
+  </si>
+  <si>
+    <t>https://www.udemy.com/course/learn-animation</t>
+  </si>
+  <si>
+    <t>Becoming a great designer is about much more than taking a single course or attending a single bootcamp.
+You have to be self-sufficient. You have to be hungry to learn.
+Throughout design school I collected every resource I found to be useful. Since then I have continued to amass a collection of links, books, articles, and more that will help you speed boost your career.</t>
+  </si>
+  <si>
+    <t>Graphic design is all around us, in a myriad of forms, both on screen and in print, yet it is always made up of images and words to create a communication goal. This four-course sequence exposes students to the fundamental skills required to make sophisticated graphic design: process, historical context, and communication through image-making and typography. The sequence is completed by a capstone project that applies the skills of each course and peer feedback in a finished branding project suitable for a professional portfolio.</t>
+  </si>
+  <si>
+    <t>Explore the essentials of visual design, from key elements and principles to its history and evolution.</t>
+  </si>
+  <si>
+    <t>Learn the theory, principles and practices involved in graphic design with this free online Graphic Design course.</t>
+  </si>
+  <si>
+    <t>Learn about the elements and principles that create good visual design</t>
+  </si>
+  <si>
+    <t>Wondering what goes into the creation of a successful design piece? Learn what are the principles of design, see examples of principles of design, and more!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">So you want to be a graphic designer? Welcome to this Graphic Design Basics course, which will teach you everything you need to know to get started. </t>
+  </si>
+  <si>
+    <t>Colors are a powerful visual tool that can help us evoke certain emotions. In this course, you’ll learn all about the fundamentals of color theory that can help you create your own color palette.</t>
+  </si>
+  <si>
+    <t>Master Graphic Design &amp; Branding Skills.
+Learn design principles, branding, and motion to create professional, portfolio-ready projects</t>
+  </si>
+  <si>
+    <t>In this 1 hour and 11 minute tutorial, Aaron Blaise will take you through the very basics of creating images in Photoshop using his methods. This Photoshop Illustration Tutorial is perfect for beginners and aspiring digital artists.
+NOTE: While the software demonstrated is Adobe Photoshop, the techniques shown here generally apply to all digital painting Apps including, Procreate, Krita, Clip Studo Paint, Corel Painter and many more.</t>
+  </si>
+  <si>
+    <t>This Reddit post outlines animation skills and several animation courses.</t>
+  </si>
+  <si>
+    <t>Alan Becker highlights each of the 12 Principles of Animation as described by Frank Thomas and Ollie Johnston in their book "The Illusion of Life."</t>
+  </si>
+  <si>
+    <t>The 12 Principles help to make your animations feel both realistic and engaging. In this series of videos we'll explore the principles one by one to show how you can apply them to your animation or motion graphics projects.</t>
+  </si>
+  <si>
+    <t>In this compilation course we'll learn everything you need to know to start animating. Well cover everything from creating a script to recording audio, all the way through to animation tips and tricks. This isn't a video about 'how to animate' so to speak, although there are plenty of those on the channel, this is a video about the process behind making your animation from start to finish. Let's get right to it</t>
+  </si>
+  <si>
+    <t>This Animatron University "Beginner" course is specifically designed for the beginner in mind. In this in depth course you'll learn how make animations with absolutely zero background in animation or design or coding. Learn HOW TO use this FREE Online tool, ANIMATRON to create fun, easy, and exciting HTML5,gifs and short animations that you can share with the WORLD!</t>
+  </si>
+  <si>
+    <t>In this course I will guide you through the process of making an animated short movie, step by step.</t>
+  </si>
+  <si>
+    <t>New to animation? Looking for a new workflow? Before you start investing in courses or software, maybe I can help! This course briefly overviews all the animation software I currently teach: Moho, Animate, After Effects and Character Animator. Which software is the easiest to use? Which provides the best bone system? Or what about frame-by-frame? This course covers these questions and offers resources to learn more, if you wish.</t>
+  </si>
+  <si>
+    <t>Pixar in a Box is a behind-the-scenes look at how Pixar artists do their jobs. You will be able to animate bouncing balls, build a swarm of robots, and make virtual fireworks explode. The subjects you learn in school — math, science, computer science, and humanities — are used every day to create amazing movies at Pixar.</t>
+  </si>
+  <si>
+    <t>Want to learn animation online for free? This course teaches you how animation actually works. You'll understand the core principles that make characters move believably, objects feel weighted, and scenes come alive. This free animation course gives you the foundation every animator needs, whether you're sketching stick figures or dreaming of working at Pixar.</t>
+  </si>
+  <si>
+    <t>Adobe After Effects is a powerful tool for motion graphics and visual effects. It can be used on its own to create stand-alone videos and animations or integrated into video editing programs like Premiere Pro. 
+In this free class, you’ll get a healthy taste of the power of After Effects as an animation and effects tool. We’ll be creating a motion graphics animation using photos and video and then use the tracking and compositing features of the program to recreate an effect from a well-known Hollywood movie.</t>
   </si>
 </sst>
 </file>
@@ -830,40 +895,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="30">
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1254,6 +1292,33 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1268,56 +1333,64 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{29CE4B51-B891-4FED-B6CE-0832EE7B1EAC}" name="Table1" displayName="Table1" ref="A1:H27" totalsRowShown="0" dataDxfId="29">
-  <autoFilter ref="A1:H27" xr:uid="{29CE4B51-B891-4FED-B6CE-0832EE7B1EAC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{29CE4B51-B891-4FED-B6CE-0832EE7B1EAC}" name="Table1" displayName="Table1" ref="A1:H27" totalsRowShown="0" dataDxfId="20">
+  <autoFilter ref="A1:H27" xr:uid="{29CE4B51-B891-4FED-B6CE-0832EE7B1EAC}">
+    <filterColumn colId="4">
+      <filters blank="1"/>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{3DBB28DD-33B7-4042-B7F3-B5060E89F664}" name="ID" dataDxfId="28">
+    <tableColumn id="1" xr3:uid="{3DBB28DD-33B7-4042-B7F3-B5060E89F664}" name="ID" dataDxfId="19">
       <calculatedColumnFormula>ROW()-1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{1F2E0A47-3518-43B8-ACAD-F8AA9B3FA0C2}" name="Course" dataDxfId="27"/>
-    <tableColumn id="8" xr3:uid="{08E04412-D137-43F6-90C3-6274D8F1475F}" name="Provider" dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{EA2CEA01-9D57-4566-BB51-937CB5EF4C8B}" name="Link" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{44826D80-7922-4F2C-A047-A6EBCDA411EA}" name="Description" dataDxfId="24"/>
-    <tableColumn id="7" xr3:uid="{2D68A384-0B4A-4939-A697-890425BBF268}" name="Hours" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{F8C7365D-FC52-4C24-B91E-8694A3EEBDDB}" name="Cost" dataDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{0D93BA61-F758-4D55-AE78-A86CE5502B5E}" name="Level" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{1F2E0A47-3518-43B8-ACAD-F8AA9B3FA0C2}" name="Course" dataDxfId="18"/>
+    <tableColumn id="8" xr3:uid="{08E04412-D137-43F6-90C3-6274D8F1475F}" name="Provider" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{EA2CEA01-9D57-4566-BB51-937CB5EF4C8B}" name="Link" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{44826D80-7922-4F2C-A047-A6EBCDA411EA}" name="Description" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{2D68A384-0B4A-4939-A697-890425BBF268}" name="Hours" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{F8C7365D-FC52-4C24-B91E-8694A3EEBDDB}" name="Cost" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{0D93BA61-F758-4D55-AE78-A86CE5502B5E}" name="Level" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C303FFE5-8D98-417D-880E-DB85C92CB383}" name="Table14" displayName="Table14" ref="A1:H16" totalsRowShown="0" dataDxfId="8">
-  <autoFilter ref="A1:H16" xr:uid="{29CE4B51-B891-4FED-B6CE-0832EE7B1EAC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{C303FFE5-8D98-417D-880E-DB85C92CB383}" name="Table14" displayName="Table14" ref="A1:H16" totalsRowShown="0" dataDxfId="29">
+  <autoFilter ref="A1:H16" xr:uid="{29CE4B51-B891-4FED-B6CE-0832EE7B1EAC}">
+    <filterColumn colId="4">
+      <filters blank="1"/>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{0227205A-05FB-49D8-9DB7-06580FAEFD61}" name="ID" dataDxfId="7">
+    <tableColumn id="1" xr3:uid="{0227205A-05FB-49D8-9DB7-06580FAEFD61}" name="ID" dataDxfId="28">
       <calculatedColumnFormula>ROW()-1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{30135BFE-F58A-462A-8C45-82F4C336217D}" name="Course" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{96FBC0EA-9DF0-4D17-A7EB-7E4095E2DFE5}" name="Provider" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{C01A10B6-88E6-4569-A16A-EDA93A283455}" name="Link" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{5FC3D772-8E9C-45C6-80F7-9A3456D7BE62}" name="Description" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{A9D41824-33F8-4A21-A318-1A7CEED0E54C}" name="Hours" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{7D5F93A2-6D53-45E3-99F7-AEC388991D3B}" name="Cost" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{964EDD01-5F45-4432-804F-4380823DEAD0}" name="Level" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{30135BFE-F58A-462A-8C45-82F4C336217D}" name="Course" dataDxfId="27"/>
+    <tableColumn id="8" xr3:uid="{96FBC0EA-9DF0-4D17-A7EB-7E4095E2DFE5}" name="Provider" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{C01A10B6-88E6-4569-A16A-EDA93A283455}" name="Link" dataDxfId="25"/>
+    <tableColumn id="6" xr3:uid="{5FC3D772-8E9C-45C6-80F7-9A3456D7BE62}" name="Description" dataDxfId="24"/>
+    <tableColumn id="7" xr3:uid="{A9D41824-33F8-4A21-A318-1A7CEED0E54C}" name="Hours" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{7D5F93A2-6D53-45E3-99F7-AEC388991D3B}" name="Cost" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{964EDD01-5F45-4432-804F-4380823DEAD0}" name="Level" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{99710536-DB71-4E03-8400-B3BDA29FD654}" name="Table2" displayName="Table2" ref="A1:G9" totalsRowShown="0" headerRowDxfId="20" dataDxfId="18" headerRowBorderDxfId="19" tableBorderDxfId="17" totalsRowBorderDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{99710536-DB71-4E03-8400-B3BDA29FD654}" name="Table2" displayName="Table2" ref="A1:G9" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8" totalsRowBorderDxfId="7">
   <autoFilter ref="A1:G9" xr:uid="{99710536-DB71-4E03-8400-B3BDA29FD654}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{E134F453-3806-43C4-8FDF-00389ABDC66E}" name="ID" dataDxfId="15">
+    <tableColumn id="1" xr3:uid="{E134F453-3806-43C4-8FDF-00389ABDC66E}" name="ID" dataDxfId="6">
       <calculatedColumnFormula>ROW()-1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{F5C13FF2-C72D-4500-AB55-A3687C29C9CB}" name="Course" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{5F865AA1-F175-4BE3-9CC1-280847A1B94F}" name="Link" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{7F5E2FFB-0415-4D23-A91F-D18147C0C87B}" name="Description" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{03D122FD-861D-4616-BC54-F434977F7341}" name="Hours" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{583253DF-20DD-4C32-A034-0A223219C6AA}" name="Cost" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{3B19AF21-D796-4E6D-B368-920BCCFDE861}" name="Level" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{F5C13FF2-C72D-4500-AB55-A3687C29C9CB}" name="Course" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{5F865AA1-F175-4BE3-9CC1-280847A1B94F}" name="Link" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{7F5E2FFB-0415-4D23-A91F-D18147C0C87B}" name="Description" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{03D122FD-861D-4616-BC54-F434977F7341}" name="Hours" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{583253DF-20DD-4C32-A034-0A223219C6AA}" name="Cost" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{3B19AF21-D796-4E6D-B368-920BCCFDE861}" name="Level" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1618,7 +1691,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <f t="shared" ref="A2:A25" si="0">ROW()-1</f>
         <v>1</v>
@@ -1645,7 +1718,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -1672,7 +1745,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -1699,7 +1772,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1726,7 +1799,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1753,7 +1826,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1780,7 +1853,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1807,7 +1880,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1834,7 +1907,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1861,7 +1934,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1888,7 +1961,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1915,7 +1988,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1942,7 +2015,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1969,7 +2042,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1996,7 +2069,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -2023,7 +2096,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -2047,7 +2120,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A18">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -2060,6 +2133,9 @@
       </c>
       <c r="D18" t="s">
         <v>89</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>156</v>
       </c>
       <c r="G18" t="s">
         <v>6</v>
@@ -2082,6 +2158,9 @@
       <c r="D19" t="s">
         <v>91</v>
       </c>
+      <c r="E19" t="s">
+        <v>157</v>
+      </c>
       <c r="F19">
         <v>11</v>
       </c>
@@ -2092,7 +2171,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -2105,6 +2184,9 @@
       </c>
       <c r="D20" t="s">
         <v>94</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>158</v>
       </c>
       <c r="F20">
         <v>2.5</v>
@@ -2130,6 +2212,9 @@
       <c r="D21" t="s">
         <v>96</v>
       </c>
+      <c r="E21" t="s">
+        <v>159</v>
+      </c>
       <c r="G21" t="s">
         <v>6</v>
       </c>
@@ -2151,6 +2236,9 @@
       <c r="D22" t="s">
         <v>99</v>
       </c>
+      <c r="E22" t="s">
+        <v>160</v>
+      </c>
       <c r="F22">
         <v>1</v>
       </c>
@@ -2175,6 +2263,9 @@
       <c r="D23" t="s">
         <v>101</v>
       </c>
+      <c r="E23" t="s">
+        <v>161</v>
+      </c>
       <c r="F23">
         <v>1</v>
       </c>
@@ -2185,7 +2276,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24">
         <f t="shared" si="0"/>
         <v>23</v>
@@ -2199,6 +2290,9 @@
       <c r="D24" t="s">
         <v>104</v>
       </c>
+      <c r="E24" s="4" t="s">
+        <v>162</v>
+      </c>
       <c r="F24">
         <v>1</v>
       </c>
@@ -2223,6 +2317,9 @@
       <c r="D25" t="s">
         <v>105</v>
       </c>
+      <c r="E25" t="s">
+        <v>163</v>
+      </c>
       <c r="F25">
         <v>1</v>
       </c>
@@ -2233,22 +2330,24 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A26" s="17">
+    <row r="26" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A26">
         <f>ROW()-1</f>
         <v>25</v>
       </c>
-      <c r="B26" s="17" t="s">
-        <v>124</v>
-      </c>
-      <c r="C26" s="17" t="s">
+      <c r="B26" t="s">
+        <v>122</v>
+      </c>
+      <c r="C26" t="s">
         <v>61</v>
       </c>
-      <c r="D26" s="17" t="s">
-        <v>125</v>
-      </c>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17">
+      <c r="D26" t="s">
+        <v>123</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="F26">
         <v>80</v>
       </c>
       <c r="G26" t="s">
@@ -2258,27 +2357,29 @@
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A27" s="17">
+    <row r="27" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A27">
         <v>26</v>
       </c>
-      <c r="B27" s="17" t="s">
+      <c r="B27" t="s">
+        <v>133</v>
+      </c>
+      <c r="C27" t="s">
+        <v>134</v>
+      </c>
+      <c r="D27" s="17" t="s">
         <v>135</v>
       </c>
-      <c r="C27" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="D27" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="E27" s="17"/>
-      <c r="F27" s="17">
+      <c r="E27" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="F27">
         <v>1</v>
       </c>
-      <c r="G27" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="H27" s="17" t="s">
+      <c r="G27" t="s">
+        <v>6</v>
+      </c>
+      <c r="H27" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2286,10 +2387,11 @@
   <hyperlinks>
     <hyperlink ref="D8" r:id="rId1" xr:uid="{4EE6C6D9-59FB-4776-802F-E8A4C652FF11}"/>
     <hyperlink ref="D9" r:id="rId2" xr:uid="{2652899C-892D-4B47-9C71-52D1D7B5701A}"/>
+    <hyperlink ref="D27" r:id="rId3" xr:uid="{A1F11D19-3FFF-40F8-82B3-83E34693A5E5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2328,7 +2430,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <f t="shared" ref="A2" si="0">ROW()-1</f>
         <v>1</v>
@@ -2355,368 +2457,394 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="17">
-        <f>ROW()-1</f>
+    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <f t="shared" ref="A3:A16" si="1">ROW()-1</f>
         <v>2</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" t="s">
         <v>110</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" t="s">
         <v>95</v>
       </c>
-      <c r="D3" s="17" t="s">
+      <c r="D3" t="s">
         <v>111</v>
       </c>
-      <c r="E3" s="17" t="s">
+      <c r="E3" t="s">
         <v>112</v>
       </c>
-      <c r="F3" s="17">
+      <c r="F3">
         <v>2.25</v>
       </c>
-      <c r="G3" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="H3" s="17" t="s">
+      <c r="G3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="17">
-        <f>ROW()-1</f>
+    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" t="s">
         <v>114</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" t="s">
         <v>98</v>
       </c>
       <c r="D4" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E4" t="s">
         <v>115</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="F4">
+        <v>4.5</v>
+      </c>
+      <c r="G4" t="s">
         <v>116</v>
       </c>
-      <c r="F4" s="17">
-        <v>4.5</v>
-      </c>
-      <c r="G4" s="17" t="s">
+      <c r="H4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
         <v>117</v>
       </c>
-      <c r="H4" s="17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="17">
-        <f>ROW()-1</f>
-        <v>4</v>
-      </c>
-      <c r="B5" s="17" t="s">
+      <c r="C5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>155</v>
+      </c>
+      <c r="E5" t="s">
+        <v>118</v>
+      </c>
+      <c r="F5">
+        <v>1.5</v>
+      </c>
+      <c r="G5" t="s">
+        <v>116</v>
+      </c>
+      <c r="H5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D6" t="s">
         <v>119</v>
       </c>
-      <c r="C5" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="D5" s="17" t="s">
-        <v>118</v>
-      </c>
-      <c r="E5" s="17" t="s">
-        <v>120</v>
-      </c>
-      <c r="F5" s="17">
-        <v>1.5</v>
-      </c>
-      <c r="G5" s="17" t="s">
-        <v>117</v>
-      </c>
-      <c r="H5" s="17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="17">
-        <f>ROW()-1</f>
-        <v>5</v>
-      </c>
-      <c r="B6" s="17" t="s">
-        <v>122</v>
-      </c>
-      <c r="C6" s="17" t="s">
-        <v>61</v>
-      </c>
-      <c r="D6" s="17" t="s">
+      <c r="E6" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="F6" s="17">
+      <c r="F6">
         <v>80</v>
       </c>
       <c r="G6" t="s">
         <v>83</v>
       </c>
-      <c r="H6" s="17" t="s">
+      <c r="H6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="17">
-        <f>ROW()-1</f>
-        <v>6</v>
-      </c>
-      <c r="B7" s="17" t="s">
+      <c r="A7">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C7" t="s">
+        <v>125</v>
+      </c>
+      <c r="D7" t="s">
         <v>126</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="E7" t="s">
+        <v>166</v>
+      </c>
+      <c r="F7">
+        <v>0.5</v>
+      </c>
+      <c r="G7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
         <v>127</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="C8" t="s">
         <v>128</v>
       </c>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17">
+      <c r="D8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E8" t="s">
+        <v>167</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8" t="s">
+        <v>6</v>
+      </c>
+      <c r="H8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>130</v>
+      </c>
+      <c r="C9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D9" t="s">
+        <v>132</v>
+      </c>
+      <c r="E9" t="s">
+        <v>168</v>
+      </c>
+      <c r="F9">
         <v>0.5</v>
       </c>
-      <c r="G7" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="H7" s="17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="17">
-        <f>ROW()-1</f>
-        <v>7</v>
-      </c>
-      <c r="B8" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="C8" s="17" t="s">
-        <v>130</v>
-      </c>
-      <c r="D8" s="17" t="s">
-        <v>131</v>
-      </c>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17">
+      <c r="G9" t="s">
+        <v>6</v>
+      </c>
+      <c r="H9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>136</v>
+      </c>
+      <c r="C10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D10" t="s">
+        <v>138</v>
+      </c>
+      <c r="E10" t="s">
+        <v>169</v>
+      </c>
+      <c r="F10">
         <v>1</v>
       </c>
-      <c r="G8" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="H8" s="17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="17">
-        <f>ROW()-1</f>
-        <v>8</v>
-      </c>
-      <c r="B9" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="C9" s="17" t="s">
-        <v>133</v>
-      </c>
-      <c r="D9" s="17" t="s">
-        <v>134</v>
-      </c>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17">
-        <v>0.5</v>
-      </c>
-      <c r="G9" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="H9" s="17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="17">
-        <f>ROW()-1</f>
-        <v>9</v>
-      </c>
-      <c r="B10" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="C10" s="17" t="s">
+      <c r="G10" t="s">
+        <v>6</v>
+      </c>
+      <c r="H10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
         <v>139</v>
       </c>
-      <c r="D10" s="17" t="s">
+      <c r="C11" t="s">
+        <v>98</v>
+      </c>
+      <c r="D11" t="s">
         <v>140</v>
       </c>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17">
+      <c r="E11" t="s">
+        <v>170</v>
+      </c>
+      <c r="F11">
+        <v>6</v>
+      </c>
+      <c r="G11" t="s">
+        <v>6</v>
+      </c>
+      <c r="H11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <f t="shared" si="1"/>
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>141</v>
+      </c>
+      <c r="C12" t="s">
+        <v>98</v>
+      </c>
+      <c r="D12" t="s">
+        <v>142</v>
+      </c>
+      <c r="E12" t="s">
+        <v>171</v>
+      </c>
+      <c r="F12">
+        <v>2</v>
+      </c>
+      <c r="G12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <f t="shared" si="1"/>
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>143</v>
+      </c>
+      <c r="C13" t="s">
+        <v>98</v>
+      </c>
+      <c r="D13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="F13">
         <v>1</v>
       </c>
-      <c r="G10" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="H10" s="17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="17">
-        <f>ROW()-1</f>
-        <v>10</v>
-      </c>
-      <c r="B11" s="17" t="s">
-        <v>141</v>
-      </c>
-      <c r="C11" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="D11" s="17" t="s">
-        <v>142</v>
-      </c>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17">
-        <v>6</v>
-      </c>
-      <c r="G11" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="H11" s="17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="17">
-        <f>ROW()-1</f>
-        <v>11</v>
-      </c>
-      <c r="B12" s="17" t="s">
-        <v>143</v>
-      </c>
-      <c r="C12" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="D12" s="17" t="s">
-        <v>144</v>
-      </c>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17">
-        <v>2</v>
-      </c>
-      <c r="G12" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="H12" s="17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="17">
-        <f>ROW()-1</f>
-        <v>12</v>
-      </c>
-      <c r="B13" s="17" t="s">
+      <c r="G13" t="s">
+        <v>6</v>
+      </c>
+      <c r="H13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <f t="shared" si="1"/>
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
         <v>145</v>
       </c>
-      <c r="C13" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="D13" s="17" t="s">
+      <c r="C14" t="s">
         <v>146</v>
       </c>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17">
+      <c r="D14" t="s">
+        <v>147</v>
+      </c>
+      <c r="E14" t="s">
+        <v>173</v>
+      </c>
+      <c r="F14">
         <v>1</v>
       </c>
-      <c r="G13" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="H13" s="17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="17">
-        <f>ROW()-1</f>
-        <v>13</v>
-      </c>
-      <c r="B14" s="17" t="s">
-        <v>147</v>
-      </c>
-      <c r="C14" s="17" t="s">
+      <c r="G14" t="s">
+        <v>6</v>
+      </c>
+      <c r="H14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <f t="shared" si="1"/>
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>150</v>
+      </c>
+      <c r="C15" t="s">
         <v>148</v>
       </c>
-      <c r="D14" s="17" t="s">
+      <c r="D15" s="17" t="s">
         <v>149</v>
       </c>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17">
+      <c r="E15" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="F15">
         <v>1</v>
       </c>
-      <c r="G14" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="H14" s="17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="17">
-        <f>ROW()-1</f>
-        <v>14</v>
-      </c>
-      <c r="B15" s="17" t="s">
+      <c r="G15" t="s">
+        <v>6</v>
+      </c>
+      <c r="H15" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>151</v>
+      </c>
+      <c r="C16" t="s">
         <v>152</v>
       </c>
-      <c r="C15" s="17" t="s">
-        <v>150</v>
-      </c>
-      <c r="D15" s="17" t="s">
-        <v>151</v>
-      </c>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17">
+      <c r="D16" t="s">
+        <v>153</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="F16">
         <v>1</v>
       </c>
-      <c r="G15" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="H15" s="17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="17">
-        <f>ROW()-1</f>
-        <v>15</v>
-      </c>
-      <c r="B16" s="17" t="s">
-        <v>153</v>
-      </c>
-      <c r="C16" s="17" t="s">
-        <v>154</v>
-      </c>
-      <c r="D16" s="17" t="s">
-        <v>155</v>
-      </c>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17">
-        <v>1</v>
-      </c>
-      <c r="G16" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="H16" s="17" t="s">
+      <c r="G16" t="s">
+        <v>6</v>
+      </c>
+      <c r="H16" t="s">
         <v>24</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D4" r:id="rId1" xr:uid="{D7D1D8DA-96F6-4BC7-A302-42593A71E1E3}"/>
+    <hyperlink ref="D5" r:id="rId2" xr:uid="{4EA0DE51-5F5D-4F6E-9FA3-B15CE77D2C7D}"/>
+    <hyperlink ref="D15" r:id="rId3" xr:uid="{9CCF8D7C-DEDA-4725-BAE9-F93B167953BF}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId4"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>